<commit_message>
fix(pnl-reporting): promote corrected template authority
</commit_message>
<xml_diff>
--- a/forecast/bff/resources/PNL_REPORTING_TEMPLATE_V1.xlsx
+++ b/forecast/bff/resources/PNL_REPORTING_TEMPLATE_V1.xlsx
@@ -1992,7 +1992,7 @@
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>    1. 인건비</x:v>
+        <x:v>1. 인건비</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
         <x:v>일반관리비</x:v>
@@ -2018,7 +2018,7 @@
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
       <x:c r="A4" s="14" t="str">
-        <x:v>    2. 감가상각비</x:v>
+        <x:v>2. 감가상각비</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
         <x:v>일반관리비</x:v>
@@ -2044,7 +2044,7 @@
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>    3. 경상개발비</x:v>
+        <x:v>3. 경상개발비</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
         <x:v>일반관리비</x:v>
@@ -2070,7 +2070,7 @@
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="14" t="str">
-        <x:v>    4. 수수료</x:v>
+        <x:v>4. 수수료</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
         <x:v>일반관리비</x:v>
@@ -2096,7 +2096,7 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="24" t="str">
-        <x:v>    5. 기타</x:v>
+        <x:v>5. 기타</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
         <x:v>일반관리비</x:v>
@@ -2146,7 +2146,7 @@
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="14" t="str">
-        <x:v>        통신비</x:v>
+        <x:v>• 통신비</x:v>
       </x:c>
       <x:c r="B8" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2172,7 +2172,7 @@
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>        소모품비</x:v>
+        <x:v>• 소모품비</x:v>
       </x:c>
       <x:c r="B9" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2198,7 +2198,7 @@
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>        도서인쇄비</x:v>
+        <x:v>• 도서인쇄비</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2224,7 +2224,7 @@
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="14" t="str">
-        <x:v>        기타 잡비</x:v>
+        <x:v>• 기타 잡비</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2300,7 +2300,7 @@
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>    1. 운반비</x:v>
+        <x:v>1. 운반비</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2326,7 +2326,7 @@
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>    2. 수수료</x:v>
+        <x:v>2. 수수료</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2352,7 +2352,7 @@
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>    3. 브랜드사용료</x:v>
+        <x:v>3. 브랜드사용료</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2378,7 +2378,7 @@
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>    4. 인건비</x:v>
+        <x:v>4. 인건비</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2404,7 +2404,7 @@
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>    5. 견본비</x:v>
+        <x:v>5. 견본비</x:v>
       </x:c>
       <x:c r="B17" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2430,7 +2430,7 @@
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>    6. 대손상각</x:v>
+        <x:v>6. 대손상각</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2456,7 +2456,7 @@
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>    7. 잡비</x:v>
+        <x:v>7. 잡비</x:v>
       </x:c>
       <x:c r="B19" s="14" t="str">
         <x:v>판매비</x:v>
@@ -2482,7 +2482,7 @@
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
       <x:c r="A20" s="24" t="str">
-        <x:v>    8. 기타</x:v>
+        <x:v>8. 기타</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
         <x:v>판매비</x:v>
@@ -2532,7 +2532,7 @@
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>        포장재료비</x:v>
+        <x:v>• 포장재료비</x:v>
       </x:c>
       <x:c r="B21" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2558,7 +2558,7 @@
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
       <x:c r="A22" s="14" t="str">
-        <x:v>        보관료/창고료</x:v>
+        <x:v>• 보관료/창고료</x:v>
       </x:c>
       <x:c r="B22" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2584,7 +2584,7 @@
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>        기타 판매부대비</x:v>
+        <x:v>• 기타 판매부대비</x:v>
       </x:c>
       <x:c r="B23" s="14" t="str">
         <x:v>세부항목</x:v>
@@ -2816,7 +2816,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C2" s="24" t="str">
-        <x:v>매출액</x:v>
+        <x:v>1. 매출액</x:v>
       </x:c>
       <x:c r="D2" s="24" t="str">
         <x:v>백만원</x:v>
@@ -2848,7 +2848,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C3" s="14" t="str">
-        <x:v>매출수량</x:v>
+        <x:v>2. 매출수량</x:v>
       </x:c>
       <x:c r="D3" s="14" t="str">
         <x:v>PCS</x:v>
@@ -2880,10 +2880,10 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C4" s="14" t="str">
-        <x:v>평균 판매 단가(ASP)</x:v>
+        <x:v>3. 평균 판매 단가(ASP)</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
-        <x:v>원/PCS</x:v>
+        <x:v>원</x:v>
       </x:c>
       <x:c r="E4" s="22" t="str">
         <x:f>IF(OR(E2="",E3="",E3=0),"",E2*1000000/E3)</x:f>
@@ -2936,7 +2936,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C5" s="14" t="str">
-        <x:v>매출원가</x:v>
+        <x:v>4. 매출원가</x:v>
       </x:c>
       <x:c r="D5" s="14" t="str">
         <x:v>백만원</x:v>
@@ -2968,7 +2968,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C6" s="14" t="str">
-        <x:v>매출원가율</x:v>
+        <x:v>• 매출원가율</x:v>
       </x:c>
       <x:c r="D6" s="14" t="str">
         <x:v>%</x:v>
@@ -3024,7 +3024,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
-        <x:v>매출총이익</x:v>
+        <x:v>5. 매출총이익</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
         <x:v>백만원</x:v>
@@ -3080,7 +3080,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>매출총이익률</x:v>
+        <x:v>• 매출총이익률</x:v>
       </x:c>
       <x:c r="D8" s="14" t="str">
         <x:v>%</x:v>
@@ -3136,7 +3136,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>판매관리비</x:v>
+        <x:v>6. 판매관리비</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
         <x:v>백만원</x:v>
@@ -3168,7 +3168,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>영업이익</x:v>
+        <x:v>7. 영업이익</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
         <x:v>백만원</x:v>
@@ -3224,7 +3224,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>영업이익률</x:v>
+        <x:v>• 영업이익률</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>%</x:v>
@@ -3280,7 +3280,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>매출액</x:v>
+        <x:v>1. 매출액</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>백만원</x:v>
@@ -3312,7 +3312,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>매출수량</x:v>
+        <x:v>2. 매출수량</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>PCS</x:v>
@@ -3344,10 +3344,10 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>평균 판매 단가(ASP)</x:v>
+        <x:v>3. 평균 판매 단가(ASP)</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>원/PCS</x:v>
+        <x:v>원</x:v>
       </x:c>
       <x:c r="E14" s="22" t="str">
         <x:f>IF(OR(E12="",E13="",E13=0),"",E12*1000000/E13)</x:f>
@@ -3400,7 +3400,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>매출원가</x:v>
+        <x:v>4. 매출원가</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
         <x:v>백만원</x:v>
@@ -3432,7 +3432,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>매출원가율</x:v>
+        <x:v>• 매출원가율</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
         <x:v>%</x:v>
@@ -3488,7 +3488,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>매출총이익</x:v>
+        <x:v>5. 매출총이익</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
         <x:v>백만원</x:v>
@@ -3544,7 +3544,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>매출총이익률</x:v>
+        <x:v>• 매출총이익률</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
         <x:v>%</x:v>
@@ -3600,7 +3600,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>판매관리비</x:v>
+        <x:v>6. 판매관리비</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
         <x:v>백만원</x:v>
@@ -3632,7 +3632,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>영업이익</x:v>
+        <x:v>7. 영업이익</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
         <x:v>백만원</x:v>
@@ -3688,7 +3688,7 @@
         <x:v>8-inch</x:v>
       </x:c>
       <x:c r="C21" s="14" t="str">
-        <x:v>영업이익률</x:v>
+        <x:v>• 영업이익률</x:v>
       </x:c>
       <x:c r="D21" s="14" t="str">
         <x:v>%</x:v>
@@ -3744,7 +3744,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C22" s="24" t="str">
-        <x:v>매출액</x:v>
+        <x:v>1. 매출액</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
         <x:v>백만원</x:v>
@@ -3776,7 +3776,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>매출수량</x:v>
+        <x:v>2. 매출수량</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
         <x:v>PCS</x:v>
@@ -3808,10 +3808,10 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>평균 판매 단가(ASP)</x:v>
+        <x:v>3. 평균 판매 단가(ASP)</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
-        <x:v>원/PCS</x:v>
+        <x:v>원</x:v>
       </x:c>
       <x:c r="E24" s="22" t="str">
         <x:f>IF(OR(E22="",E23="",E23=0),"",E22*1000000/E23)</x:f>
@@ -3864,7 +3864,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C25" s="14" t="str">
-        <x:v>매출원가</x:v>
+        <x:v>4. 매출원가</x:v>
       </x:c>
       <x:c r="D25" s="14" t="str">
         <x:v>백만원</x:v>
@@ -3896,7 +3896,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>매출원가율</x:v>
+        <x:v>• 매출원가율</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
         <x:v>%</x:v>
@@ -3952,7 +3952,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>매출총이익</x:v>
+        <x:v>5. 매출총이익</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4008,7 +4008,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>매출총이익률</x:v>
+        <x:v>• 매출총이익률</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
         <x:v>%</x:v>
@@ -4064,7 +4064,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C29" s="14" t="str">
-        <x:v>판매관리비</x:v>
+        <x:v>6. 판매관리비</x:v>
       </x:c>
       <x:c r="D29" s="14" t="str">
         <x:v>백만원</x:v>
@@ -4096,7 +4096,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
-        <x:v>영업이익</x:v>
+        <x:v>7. 영업이익</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4152,7 +4152,7 @@
         <x:v>4-inch</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>영업이익률</x:v>
+        <x:v>• 영업이익률</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
         <x:v>%</x:v>
@@ -4208,7 +4208,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C32" s="24" t="str">
-        <x:v>매출액</x:v>
+        <x:v>1. 매출액</x:v>
       </x:c>
       <x:c r="D32" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4240,7 +4240,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C33" s="14" t="str">
-        <x:v>매출수량</x:v>
+        <x:v>2. 매출수량</x:v>
       </x:c>
       <x:c r="D33" s="14" t="str">
         <x:v>m</x:v>
@@ -4272,10 +4272,10 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>평균 판매 단가(ASP)</x:v>
+        <x:v>3. 평균 판매 단가(ASP)</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>원/m</x:v>
+        <x:v>원</x:v>
       </x:c>
       <x:c r="E34" s="22" t="str">
         <x:f>IF(OR(E32="",E33="",E33=0),"",E32*1000000/E33)</x:f>
@@ -4328,7 +4328,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>매출원가</x:v>
+        <x:v>4. 매출원가</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
         <x:v>백만원</x:v>
@@ -4360,7 +4360,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C36" s="14" t="str">
-        <x:v>매출원가율</x:v>
+        <x:v>• 매출원가율</x:v>
       </x:c>
       <x:c r="D36" s="14" t="str">
         <x:v>%</x:v>
@@ -4416,7 +4416,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C37" s="24" t="str">
-        <x:v>매출총이익</x:v>
+        <x:v>5. 매출총이익</x:v>
       </x:c>
       <x:c r="D37" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4472,7 +4472,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C38" s="14" t="str">
-        <x:v>매출총이익률</x:v>
+        <x:v>• 매출총이익률</x:v>
       </x:c>
       <x:c r="D38" s="14" t="str">
         <x:v>%</x:v>
@@ -4528,7 +4528,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>판매관리비</x:v>
+        <x:v>6. 판매관리비</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
         <x:v>백만원</x:v>
@@ -4560,7 +4560,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C40" s="24" t="str">
-        <x:v>영업이익</x:v>
+        <x:v>7. 영업이익</x:v>
       </x:c>
       <x:c r="D40" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4616,7 +4616,7 @@
         <x:v>LENGTH</x:v>
       </x:c>
       <x:c r="C41" s="14" t="str">
-        <x:v>영업이익률</x:v>
+        <x:v>• 영업이익률</x:v>
       </x:c>
       <x:c r="D41" s="14" t="str">
         <x:v>%</x:v>
@@ -4669,10 +4669,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B42" s="24" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C42" s="24" t="str">
-        <x:v>매출액</x:v>
+        <x:v>1. 매출액</x:v>
       </x:c>
       <x:c r="D42" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4701,10 +4701,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B43" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>매출원가</x:v>
+        <x:v>2. 매출원가</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
         <x:v>백만원</x:v>
@@ -4733,10 +4733,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B44" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C44" s="14" t="str">
-        <x:v>매출원가율</x:v>
+        <x:v>• 매출원가율</x:v>
       </x:c>
       <x:c r="D44" s="14" t="str">
         <x:v>%</x:v>
@@ -4789,10 +4789,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B45" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C45" s="24" t="str">
-        <x:v>매출총이익</x:v>
+        <x:v>3. 매출총이익</x:v>
       </x:c>
       <x:c r="D45" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4845,10 +4845,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B46" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C46" s="14" t="str">
-        <x:v>매출총이익률</x:v>
+        <x:v>• 매출총이익률</x:v>
       </x:c>
       <x:c r="D46" s="14" t="str">
         <x:v>%</x:v>
@@ -4901,10 +4901,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B47" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C47" s="14" t="str">
-        <x:v>판매관리비</x:v>
+        <x:v>4. 판매관리비</x:v>
       </x:c>
       <x:c r="D47" s="14" t="str">
         <x:v>백만원</x:v>
@@ -4933,10 +4933,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B48" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C48" s="24" t="str">
-        <x:v>영업이익</x:v>
+        <x:v>5. 영업이익</x:v>
       </x:c>
       <x:c r="D48" s="24" t="str">
         <x:v>백만원</x:v>
@@ -4989,10 +4989,10 @@
         <x:v>신사업</x:v>
       </x:c>
       <x:c r="B49" s="14" t="str">
-        <x:v>item</x:v>
+        <x:v>해당없음</x:v>
       </x:c>
       <x:c r="C49" s="14" t="str">
-        <x:v>영업이익률</x:v>
+        <x:v>• 영업이익률</x:v>
       </x:c>
       <x:c r="D49" s="14" t="str">
         <x:v>%</x:v>

</xml_diff>